<commit_message>
added list of available settings and settings access
</commit_message>
<xml_diff>
--- a/project docs/GoPro_settings_list.xlsx
+++ b/project docs/GoPro_settings_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PythonProjects\Go2Kin\project docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F940FD39-685A-4152-9B19-05610D830DD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A441B9AD-2FFE-4340-9CC4-071AB3ED6BB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12960" yWindow="105" windowWidth="38700" windowHeight="15345" xr2:uid="{25ADDBA5-24B8-4C9A-8BD6-A7499FF0E2B5}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="67">
   <si>
     <t>GoPro seettings list (Hero 12 black)</t>
   </si>
@@ -235,6 +235,9 @@
   </si>
   <si>
     <t>set to Linear (4) - just for precaution as we do not use Webcam mode</t>
+  </si>
+  <si>
+    <t>YES</t>
   </si>
 </sst>
 </file>
@@ -650,6 +653,9 @@
       <c r="C6" s="2" t="s">
         <v>44</v>
       </c>
+      <c r="F6" s="2" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="7" spans="1:7" s="2" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
@@ -756,6 +762,9 @@
       <c r="E14" s="2" t="s">
         <v>44</v>
       </c>
+      <c r="F14" s="2" t="s">
+        <v>66</v>
+      </c>
       <c r="G14" s="2" t="s">
         <v>48</v>
       </c>
@@ -770,6 +779,9 @@
       <c r="D15" s="2" t="s">
         <v>44</v>
       </c>
+      <c r="F15" s="2" t="s">
+        <v>66</v>
+      </c>
       <c r="G15" s="2" t="s">
         <v>51</v>
       </c>
@@ -854,6 +866,9 @@
       <c r="D21" s="2" t="s">
         <v>44</v>
       </c>
+      <c r="F21" s="2" t="s">
+        <v>66</v>
+      </c>
       <c r="G21" s="2" t="s">
         <v>55</v>
       </c>
@@ -1064,6 +1079,9 @@
       <c r="D36" s="2" t="s">
         <v>44</v>
       </c>
+      <c r="F36" s="2" t="s">
+        <v>66</v>
+      </c>
       <c r="G36" s="2" t="s">
         <v>62</v>
       </c>
@@ -1078,6 +1096,9 @@
       <c r="D37" s="2" t="s">
         <v>44</v>
       </c>
+      <c r="F37" s="2" t="s">
+        <v>66</v>
+      </c>
       <c r="G37" s="2" t="s">
         <v>63</v>
       </c>
@@ -1119,6 +1140,9 @@
       </c>
       <c r="D40" s="2" t="s">
         <v>44</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>66</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>64</v>

</xml_diff>